<commit_message>
Refine feature freeze business package
</commit_message>
<xml_diff>
--- a/任务规格转化.xlsx
+++ b/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R5491321870eb48e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R2f9f0bf69392457b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -367,10 +367,10 @@
     </x:row>
     <x:row r="8" ht="48" customHeight="1">
       <x:c r="A8" s="5" t="str">
-        <x:v>Helm步骤</x:v>
+        <x:v>Chart处理步骤</x:v>
       </x:c>
       <x:c r="B8" s="5" t="str">
-        <x:v>读取合同与案例，完成Chart、身份权限、网络边界、安全设置和Hook，再逐案例渲染并导出业务交接文件</x:v>
+        <x:v>读取合同与发布案例，完成Chart、身份权限、网络边界、安全设置和Hook，再逐案例渲染并导出业务交接文件</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
@@ -391,58 +391,66 @@
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
       <x:c r="A11" s="5" t="str">
-        <x:v>交付消费者</x:v>
+        <x:v>发布案例衔接</x:v>
       </x:c>
       <x:c r="B11" s="5" t="str">
-        <x:v>平台发布人员消费对象清单，安全人员消费权限清单，网络团队消费边界清单，特征治理人员消费Hook顺序和发布交接记录</x:v>
+        <x:v>预览、生产和强监管案例分别提供发布名、命名空间、values、副本、策略模式及Hook截止时间，Chart保持案例可配置</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="48" customHeight="1">
       <x:c r="A12" s="5" t="str">
-        <x:v>对象实现边界</x:v>
+        <x:v>交付消费者</x:v>
       </x:c>
       <x:c r="B12" s="5" t="str">
-        <x:v>对象名与命名空间由发布案例驱动；Deployment副本、策略模式和Job截止时间由对应values驱动；合同数据由外部JSON驱动</x:v>
+        <x:v>平台发布人员使用对象清单，安全人员复核权限清单，网络团队核对边界清单，特征治理人员依据Hook顺序和发布交接记录安排封账窗口</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="48" customHeight="1">
       <x:c r="A13" s="5" t="str">
+        <x:v>对象实现边界</x:v>
+      </x:c>
+      <x:c r="B13" s="5" t="str">
+        <x:v>对象名与命名空间由发布案例驱动；Deployment副本、策略模式和Job截止时间由对应values驱动；合同数据由外部JSON驱动</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="48" customHeight="1">
+      <x:c r="A14" s="5" t="str">
         <x:v>权限实现边界</x:v>
       </x:c>
-      <x:c r="B13" s="5" t="str">
+      <x:c r="B14" s="5" t="str">
         <x:v>Role权限等于合同集合且限于命名空间，RoleBinding只连接当前控制器ServiceAccount与Role</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="33" customHeight="1">
-      <x:c r="A14" s="5" t="str">
-        <x:v>网络实现边界</x:v>
-      </x:c>
-      <x:c r="B14" s="5" t="str">
-        <x:v>入站仅接纳合同训练编排器，出站仅允许合同集群DNS与对象存储通路</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="33" customHeight="1">
       <x:c r="A15" s="5" t="str">
-        <x:v>安全与Hook边界</x:v>
+        <x:v>网络实现边界</x:v>
       </x:c>
       <x:c r="B15" s="5" t="str">
-        <x:v>三个工作负载使用同一安全基线；两个Job按合同职责、阶段、权重和删除策略编排</x:v>
+        <x:v>入站仅接纳合同训练编排器，出站仅允许合同集群DNS与对象存储通路</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="33" customHeight="1">
       <x:c r="A16" s="5" t="str">
+        <x:v>安全与Hook边界</x:v>
+      </x:c>
+      <x:c r="B16" s="5" t="str">
+        <x:v>三个工作负载使用同一安全基线；两个Job按合同职责、阶段、权重和删除策略编排</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="33" customHeight="1">
+      <x:c r="A17" s="5" t="str">
         <x:v>报告实现边界</x:v>
       </x:c>
-      <x:c r="B16" s="5" t="str">
+      <x:c r="B17" s="5" t="str">
         <x:v>四份CSV从Helm渲染对象导出，发布交接记录汇总案例字段、对象数和四份CSV记录数</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="48" customHeight="1">
-      <x:c r="A17" s="5" t="str">
-        <x:v>实现边界</x:v>
-      </x:c>
-      <x:c r="B17" s="5" t="str">
-        <x:v>业务处理采用本地Chart渲染；发布名、命名空间、副本、策略模式和Job截止时间均由输入驱动；模板拆分和等价YAML排版可以不同</x:v>
+    <x:row r="18" ht="48" customHeight="1">
+      <x:c r="A18" s="5" t="str">
+        <x:v>配置来源边界</x:v>
+      </x:c>
+      <x:c r="B18" s="5" t="str">
+        <x:v>发布名、命名空间、副本、策略模式和Job截止时间均由本次业务输入驱动，完成Chart不得固化具体案例值</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>